<commit_message>
adding other plotting options
</commit_message>
<xml_diff>
--- a/uploads/filmlessData.xlsx
+++ b/uploads/filmlessData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\homedir-cifs.nyumc.org\eh96\apps\xp\desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/EmilyHuang/Desktop/NYU Langone/matlab/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACDDFE12-AD53-47D4-8EE3-EF2B2A4B25FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F5AAC5-5B37-0445-8669-7AF316EC456B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="705" windowWidth="21000" windowHeight="10425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="22260" windowHeight="12640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,10 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -338,9 +342,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1">
         <v>91</v>
       </c>
@@ -348,7 +352,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>93</v>
       </c>
@@ -356,7 +360,7 @@
         <v>4.3799999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>95</v>
       </c>
@@ -364,7 +368,7 @@
         <v>0.39169999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>97</v>
       </c>
@@ -372,7 +376,7 @@
         <v>0.91890000000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>99</v>
       </c>
@@ -380,7 +384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>100</v>
       </c>
@@ -388,7 +392,7 @@
         <v>0.99560000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>101</v>
       </c>
@@ -396,7 +400,7 @@
         <v>0.99609999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>103</v>
       </c>
@@ -404,7 +408,7 @@
         <v>0.95899999999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>105</v>
       </c>
@@ -412,7 +416,7 @@
         <v>0.59099999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>107</v>
       </c>
@@ -420,7 +424,7 @@
         <v>0.15290000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>109</v>
       </c>

</xml_diff>